<commit_message>
FB001-41,42,43: Login within server permission, Internal user login via IdP, Exchange IdP token to new token
</commit_message>
<xml_diff>
--- a/Documents/ManageTasks.xlsx
+++ b/Documents/ManageTasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huynhngocson/Desktop/up-skills/Fakebook/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0502CFC0-0F3A-514B-A9CE-B4B621E2C1B9}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70933857-999A-3C44-8BC3-51E658E2DF0D}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="1300" windowWidth="37820" windowHeight="19660" activeTab="2" xr2:uid="{14631E72-EE2B-0947-82C4-7D9E8B7B85EF}"/>
+    <workbookView xWindow="580" yWindow="1140" windowWidth="37820" windowHeight="19660" activeTab="3" xr2:uid="{14631E72-EE2B-0947-82C4-7D9E8B7B85EF}"/>
   </bookViews>
   <sheets>
     <sheet name="Epics" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="129">
   <si>
     <t>Description</t>
   </si>
@@ -396,13 +396,37 @@
   </si>
   <si>
     <t>SCRUM-40</t>
+  </si>
+  <si>
+    <t>SCRUM-41</t>
+  </si>
+  <si>
+    <t>SCRUM-42</t>
+  </si>
+  <si>
+    <t>Implement Internal User Login</t>
+  </si>
+  <si>
+    <t>Implement Temporary API to Exchange the new token from IdP token</t>
+  </si>
+  <si>
+    <t>[Temporary] Implement API to Exchange IdP token</t>
+  </si>
+  <si>
+    <t>SCRUM-43</t>
+  </si>
+  <si>
+    <t>[Temporary] Implement API to get User Permissions from token</t>
+  </si>
+  <si>
+    <t>Implement Temporary API to get some fake permissions to support the IdP External Login feature</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -455,8 +479,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -497,6 +529,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -613,7 +651,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -704,6 +742,9 @@
     <xf numFmtId="49" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="7" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -743,6 +784,18 @@
     <xf numFmtId="49" fontId="2" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -752,24 +805,12 @@
     <xf numFmtId="49" fontId="1" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -778,6 +819,12 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1375,12 +1422,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
     </row>
     <row r="4" spans="1:6" ht="24" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -1403,13 +1450,13 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="125" x14ac:dyDescent="0.2">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="38" t="s">
+      <c r="C5" s="39" t="s">
         <v>32</v>
       </c>
       <c r="D5" s="15" t="s">
@@ -1423,9 +1470,9 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="50" x14ac:dyDescent="0.2">
-      <c r="A6" s="39"/>
-      <c r="B6" s="37"/>
-      <c r="C6" s="38"/>
+      <c r="A6" s="40"/>
+      <c r="B6" s="38"/>
+      <c r="C6" s="39"/>
       <c r="D6" s="15" t="s">
         <v>43</v>
       </c>
@@ -1437,9 +1484,9 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="25" x14ac:dyDescent="0.2">
-      <c r="A7" s="39"/>
-      <c r="B7" s="37"/>
-      <c r="C7" s="38"/>
+      <c r="A7" s="40"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="39"/>
       <c r="D7" s="15" t="s">
         <v>44</v>
       </c>
@@ -1479,13 +1526,13 @@
       <c r="F9" s="14"/>
     </row>
     <row r="10" spans="1:6" ht="50" x14ac:dyDescent="0.2">
-      <c r="A10" s="40" t="s">
+      <c r="A10" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41" t="s">
+      <c r="C10" s="42" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="16" t="s">
@@ -1499,9 +1546,9 @@
       </c>
     </row>
     <row r="11" spans="1:6" ht="25" x14ac:dyDescent="0.2">
-      <c r="A11" s="40"/>
-      <c r="B11" s="41"/>
-      <c r="C11" s="41"/>
+      <c r="A11" s="41"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42"/>
       <c r="D11" s="16" t="s">
         <v>46</v>
       </c>
@@ -1513,13 +1560,13 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="33" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="35" t="s">
         <v>27</v>
       </c>
       <c r="D12" s="15" t="s">
@@ -1533,9 +1580,9 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="50" x14ac:dyDescent="0.2">
-      <c r="A13" s="33"/>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
+      <c r="A13" s="34"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="36"/>
       <c r="D13" s="15" t="s">
         <v>48</v>
       </c>
@@ -1654,7 +1701,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EF5C440-AD56-C140-BA37-3A80F9AAE5E1}">
-  <dimension ref="A2:F28"/>
+  <dimension ref="A2:F29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1667,12 +1714,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" ht="67" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
     </row>
     <row r="4" spans="1:6" ht="24" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -1698,10 +1745,10 @@
       <c r="A5" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="43" t="s">
         <v>88</v>
       </c>
       <c r="D5" s="20" t="s">
@@ -1716,8 +1763,8 @@
     </row>
     <row r="6" spans="1:6" ht="100" x14ac:dyDescent="0.2">
       <c r="A6" s="26"/>
-      <c r="B6" s="43"/>
-      <c r="C6" s="43"/>
+      <c r="B6" s="44"/>
+      <c r="C6" s="44"/>
       <c r="D6" s="20" t="s">
         <v>85</v>
       </c>
@@ -1730,8 +1777,8 @@
     </row>
     <row r="7" spans="1:6" ht="25" x14ac:dyDescent="0.2">
       <c r="A7" s="26"/>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
+      <c r="B7" s="44"/>
+      <c r="C7" s="44"/>
       <c r="D7" s="20" t="s">
         <v>79</v>
       </c>
@@ -1744,8 +1791,8 @@
     </row>
     <row r="8" spans="1:6" ht="25" x14ac:dyDescent="0.2">
       <c r="A8" s="26"/>
-      <c r="B8" s="43"/>
-      <c r="C8" s="43"/>
+      <c r="B8" s="44"/>
+      <c r="C8" s="44"/>
       <c r="D8" s="20" t="s">
         <v>80</v>
       </c>
@@ -1758,8 +1805,8 @@
     </row>
     <row r="9" spans="1:6" ht="25" x14ac:dyDescent="0.2">
       <c r="A9" s="27"/>
-      <c r="B9" s="44"/>
-      <c r="C9" s="44"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="45"/>
       <c r="D9" s="20" t="s">
         <v>81</v>
       </c>
@@ -1885,34 +1932,52 @@
       <c r="F16" s="19"/>
     </row>
     <row r="17" spans="1:6" ht="25" x14ac:dyDescent="0.2">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="58" t="s">
         <v>120</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="59" t="s">
         <v>118</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="59" t="s">
         <v>119</v>
       </c>
-      <c r="D17" s="21"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-    </row>
-    <row r="18" spans="1:6" ht="24" x14ac:dyDescent="0.3">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-    </row>
-    <row r="19" spans="1:6" ht="24" x14ac:dyDescent="0.3">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
+      <c r="D17" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="50" x14ac:dyDescent="0.2">
+      <c r="A18" s="58"/>
+      <c r="B18" s="59"/>
+      <c r="C18" s="59"/>
+      <c r="D18" s="32" t="s">
+        <v>122</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="F18" s="22" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="50" x14ac:dyDescent="0.2">
+      <c r="A19" s="58"/>
+      <c r="B19" s="59"/>
+      <c r="C19" s="59"/>
+      <c r="D19" s="32" t="s">
+        <v>126</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="F19" s="22" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="20" spans="1:6" ht="24" x14ac:dyDescent="0.3">
       <c r="A20" s="12"/>
@@ -1979,18 +2044,29 @@
       <c r="F27" s="12"/>
     </row>
     <row r="28" spans="1:6" ht="24" x14ac:dyDescent="0.3">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
+      <c r="A28" s="12"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+    </row>
+    <row r="29" spans="1:6" ht="24" x14ac:dyDescent="0.3">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
     <mergeCell ref="B5:B9"/>
     <mergeCell ref="C5:C9"/>
     <mergeCell ref="B2:E2"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C17:C19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2011,12 +2087,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" ht="67" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="37" t="s">
         <v>99</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
     </row>
     <row r="4" spans="1:6" ht="24" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -2039,13 +2115,13 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="50" t="s">
         <v>100</v>
       </c>
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="43" t="s">
         <v>101</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="43" t="s">
         <v>109</v>
       </c>
       <c r="D5" s="20" t="s">
@@ -2059,9 +2135,9 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="25" x14ac:dyDescent="0.2">
-      <c r="A6" s="46"/>
-      <c r="B6" s="43"/>
-      <c r="C6" s="43"/>
+      <c r="A6" s="51"/>
+      <c r="B6" s="44"/>
+      <c r="C6" s="44"/>
       <c r="D6" s="20" t="s">
         <v>104</v>
       </c>
@@ -2073,9 +2149,9 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="50" x14ac:dyDescent="0.2">
-      <c r="A7" s="47"/>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
+      <c r="A7" s="52"/>
+      <c r="B7" s="44"/>
+      <c r="C7" s="44"/>
       <c r="D7" s="20" t="s">
         <v>105</v>
       </c>
@@ -2087,13 +2163,13 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="50" x14ac:dyDescent="0.2">
-      <c r="A8" s="48" t="s">
+      <c r="A8" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="B8" s="51" t="s">
+      <c r="B8" s="48" t="s">
         <v>56</v>
       </c>
-      <c r="C8" s="54" t="s">
+      <c r="C8" s="55" t="s">
         <v>110</v>
       </c>
       <c r="D8" s="21" t="s">
@@ -2107,9 +2183,9 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="25" x14ac:dyDescent="0.2">
-      <c r="A9" s="49"/>
-      <c r="B9" s="52"/>
-      <c r="C9" s="55"/>
+      <c r="A9" s="53"/>
+      <c r="B9" s="54"/>
+      <c r="C9" s="56"/>
       <c r="D9" s="21" t="s">
         <v>107</v>
       </c>
@@ -2121,9 +2197,9 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="50" x14ac:dyDescent="0.2">
-      <c r="A10" s="50"/>
-      <c r="B10" s="53"/>
-      <c r="C10" s="56"/>
+      <c r="A10" s="47"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="57"/>
       <c r="D10" s="21" t="s">
         <v>108</v>
       </c>

</xml_diff>